<commit_message>
Correciones PMAX y Módulos
</commit_message>
<xml_diff>
--- a/Areas_Paises.xlsx
+++ b/Areas_Paises.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta.sharepoint.com/sites/BIPOWER/Shared Documents/General/Distribución Atenea/Codigos/Distribución OBS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{A8E03CFD-D3C2-4BD9-85BF-A581898274A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A734805F-411F-45BD-8C1A-006D80213915}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{A8E03CFD-D3C2-4BD9-85BF-A581898274A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{303007D5-4197-4F40-AB0E-69720AB92626}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{996CFF7E-4120-45EC-B5A3-4D8213062A4C}"/>
   </bookViews>
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Paises!$P$1:$V$225</definedName>
     <definedName name="PAISES">Paises!$A$1:$B$17</definedName>
     <definedName name="PILAR">Paises!$AF$1:$AG$18</definedName>
-    <definedName name="PROGRAMAS">Areas!$A$1:$G$46</definedName>
+    <definedName name="PROGRAMAS">Areas!$A$1:$G$47</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1440" uniqueCount="560">
   <si>
     <t>PROGRAMA</t>
   </si>
@@ -1723,6 +1723,9 @@
   </si>
   <si>
     <t>COMERCIO</t>
+  </si>
+  <si>
+    <t>Máster de Formación Permanente en Marketing Digital, E-commerce e Inteligencia Artificial</t>
   </si>
 </sst>
 </file>
@@ -2346,29 +2349,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 4" xfId="2" xr:uid="{625F2583-C0A4-468A-84E4-A45687601707}"/>
   </cellStyles>
-  <dxfs count="47">
-    <dxf>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="45">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3724,6 +3705,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="PROGRAMAS"/>
@@ -6597,6 +6579,247 @@
           </cell>
           <cell r="C358" t="str">
             <v>IA</v>
+          </cell>
+        </row>
+        <row r="359">
+          <cell r="B359" t="str">
+            <v>Máster de Dirección Permanente en Dirección y Automatización Industrial</v>
+          </cell>
+          <cell r="C359" t="str">
+            <v>PROD</v>
+          </cell>
+        </row>
+        <row r="360">
+          <cell r="B360" t="str">
+            <v>Máster de formación Permanente en Coaching directivo y liderazgo</v>
+          </cell>
+          <cell r="C360" t="str">
+            <v>COACH</v>
+          </cell>
+        </row>
+        <row r="361">
+          <cell r="B361" t="str">
+            <v>Máster de Formación permanente en Coaching diretivo y liderazgo</v>
+          </cell>
+          <cell r="C361" t="str">
+            <v>COACH</v>
+          </cell>
+        </row>
+        <row r="362">
+          <cell r="B362" t="str">
+            <v>Máster de Formación Permanente en Direcció de Marketing y Gestión Comercial</v>
+          </cell>
+          <cell r="C362" t="str">
+            <v>MKT GC</v>
+          </cell>
+        </row>
+        <row r="363">
+          <cell r="B363" t="str">
+            <v xml:space="preserve">Máster de Formación permanente en Marketing Digital, eCommerce e Inteligencia Artificial </v>
+          </cell>
+          <cell r="C363" t="str">
+            <v>MKT EC</v>
+          </cell>
+        </row>
+        <row r="364">
+          <cell r="B364" t="str">
+            <v>Máster de formación permanente en Project Management</v>
+          </cell>
+          <cell r="C364" t="str">
+            <v>PM ESP</v>
+          </cell>
+        </row>
+        <row r="365">
+          <cell r="B365" t="str">
+            <v>Máster de Formación Permanente en Supply Chain Management</v>
+          </cell>
+          <cell r="C365" t="str">
+            <v>SUPPLY</v>
+          </cell>
+        </row>
+        <row r="366">
+          <cell r="B366" t="str">
+            <v>Máster en  Ciberseguridad</v>
+          </cell>
+          <cell r="C366" t="str">
+            <v>CIBER</v>
+          </cell>
+        </row>
+        <row r="367">
+          <cell r="B367" t="str">
+            <v>Máster en Direccción de sistemas de la información</v>
+          </cell>
+          <cell r="C367" t="str">
+            <v>SISTEM</v>
+          </cell>
+        </row>
+        <row r="368">
+          <cell r="B368" t="str">
+            <v xml:space="preserve">Máster en Dirección de Comunicación </v>
+          </cell>
+          <cell r="C368" t="str">
+            <v>COMUNIC</v>
+          </cell>
+        </row>
+        <row r="369">
+          <cell r="B369" t="str">
+            <v>Máster en n Transformación Digital</v>
+          </cell>
+          <cell r="C369" t="str">
+            <v>TR DIGI</v>
+          </cell>
+        </row>
+        <row r="370">
+          <cell r="B370" t="str">
+            <v>Máster de Formación Permanente en Dirección de la Producción y Automatización Industrial -</v>
+          </cell>
+          <cell r="C370" t="str">
+            <v>PROD</v>
+          </cell>
+        </row>
+        <row r="371">
+          <cell r="B371" t="str">
+            <v xml:space="preserve">Máster en derecho internacional de la empresa </v>
+          </cell>
+          <cell r="C371" t="str">
+            <v>DERECHO</v>
+          </cell>
+        </row>
+        <row r="372">
+          <cell r="B372" t="str">
+            <v>Máster de Formación Permanente en Neuromarketing y comportamiento del consumidor</v>
+          </cell>
+          <cell r="C372" t="str">
+            <v>NEURO MKT</v>
+          </cell>
+        </row>
+        <row r="373">
+          <cell r="B373" t="str">
+            <v>Máster de Formación Permanente en Neuromarketing y Comportamiento del Consumidor</v>
+          </cell>
+          <cell r="C373" t="str">
+            <v>NEURO MKT</v>
+          </cell>
+        </row>
+        <row r="374">
+          <cell r="B374" t="str">
+            <v xml:space="preserve"> Máster de Formación Permanente en Neuromarketing y comportamiento del consumidor</v>
+          </cell>
+          <cell r="C374" t="str">
+            <v>NEURO MKT</v>
+          </cell>
+        </row>
+        <row r="375">
+          <cell r="B375" t="str">
+            <v xml:space="preserve">Máster de Formación Permanente en Neuromarketing y comportamiento del consumidor </v>
+          </cell>
+          <cell r="C375" t="str">
+            <v>NEURO MKT</v>
+          </cell>
+        </row>
+        <row r="376">
+          <cell r="B376" t="str">
+            <v>Lifelong Digital Marketing, E-Commerce and Artificial Intelligence</v>
+          </cell>
+          <cell r="C376" t="str">
+            <v>MKT EC</v>
+          </cell>
+        </row>
+        <row r="377">
+          <cell r="B377" t="str">
+            <v>Máster de Dirección Financiera</v>
+          </cell>
+          <cell r="C377" t="str">
+            <v>FINANC</v>
+          </cell>
+        </row>
+        <row r="378">
+          <cell r="B378" t="str">
+            <v>Máster de Formación Permanente en Branding y Estrategia de Marca -</v>
+          </cell>
+          <cell r="C378" t="str">
+            <v>BRAND</v>
+          </cell>
+        </row>
+        <row r="379">
+          <cell r="B379" t="str">
+            <v>Máster en Diección Estratégica de Operaciones e Innovación</v>
+          </cell>
+          <cell r="C379" t="str">
+            <v>OPER</v>
+          </cell>
+        </row>
+        <row r="380">
+          <cell r="B380" t="str">
+            <v>Máster en Fintech e innovación financiera</v>
+          </cell>
+          <cell r="C380" t="str">
+            <v>FINTECH</v>
+          </cell>
+        </row>
+        <row r="381">
+          <cell r="B381" t="str">
+            <v>Máster de Formación Permanente en Marketing Digital, E-commerce e Inteligencia Artificial</v>
+          </cell>
+          <cell r="C381" t="str">
+            <v>MKT EC</v>
+          </cell>
+        </row>
+        <row r="382">
+          <cell r="B382" t="str">
+            <v>Máster de Formación Permanente en  Customer Experience Management</v>
+          </cell>
+          <cell r="C382" t="str">
+            <v>CX</v>
+          </cell>
+        </row>
+        <row r="383">
+          <cell r="B383" t="str">
+            <v>Máster de Formación Permanente en Business Intelligence &amp; Data Analytics</v>
+          </cell>
+          <cell r="C383" t="str">
+            <v>BI</v>
+          </cell>
+        </row>
+        <row r="384">
+          <cell r="B384" t="str">
+            <v>Máster de Formación Permanente en Coaching, Liderazgo Directivo e Inteligencia Emocional</v>
+          </cell>
+          <cell r="C384" t="str">
+            <v>COACH</v>
+          </cell>
+        </row>
+        <row r="385">
+          <cell r="B385" t="str">
+            <v>Marketing Digital, eCommerce e
+Inteligencia Artificial</v>
+          </cell>
+          <cell r="C385" t="str">
+            <v>MKT EC</v>
+          </cell>
+        </row>
+        <row r="386">
+          <cell r="B386" t="str">
+            <v>Máster de Formación Permanente en Responsabilidad Social Corporativa y Liderazgo Sostenibl</v>
+          </cell>
+          <cell r="C386" t="str">
+            <v>RSC</v>
+          </cell>
+        </row>
+        <row r="387">
+          <cell r="B387" t="str">
+            <v>Máster de Formación Permanente en Supply Chain Management y Logística -</v>
+          </cell>
+          <cell r="C387" t="str">
+            <v>SUPPLY</v>
+          </cell>
+        </row>
+        <row r="388">
+          <cell r="B388" t="str">
+            <v>Máster en Business Intelligence &amp; Data Analytics</v>
+          </cell>
+          <cell r="C388" t="str">
+            <v>BI</v>
           </cell>
         </row>
       </sheetData>
@@ -14907,128 +15130,128 @@
     <mergeCell ref="BH32:BH41"/>
   </mergeCells>
   <conditionalFormatting sqref="A28:A30 A43:A1048576 A1:A26">
-    <cfRule type="duplicateValues" dxfId="46" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D357:D1048576 D1:D351">
-    <cfRule type="duplicateValues" dxfId="45" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P42">
-    <cfRule type="duplicateValues" dxfId="44" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P180">
-    <cfRule type="duplicateValues" dxfId="43" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P193:P194">
-    <cfRule type="duplicateValues" dxfId="42" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P196:P198">
-    <cfRule type="duplicateValues" dxfId="41" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P199">
-    <cfRule type="duplicateValues" dxfId="40" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P204">
-    <cfRule type="duplicateValues" dxfId="39" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P208">
-    <cfRule type="duplicateValues" dxfId="38" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P209">
-    <cfRule type="duplicateValues" dxfId="37" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P216 P195 P181:P184 P191:P192 P200:P203 P205:P207 P211:P212 P218:P1048576 P43:P68 P1:P11 P40 P73:P146 P13:P38 P70:P71 P148:P179">
-    <cfRule type="duplicateValues" dxfId="36" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P217">
-    <cfRule type="duplicateValues" dxfId="35" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P210:Q210">
-    <cfRule type="duplicateValues" dxfId="34" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q46">
-    <cfRule type="duplicateValues" dxfId="33" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q47">
-    <cfRule type="duplicateValues" dxfId="32" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q117">
-    <cfRule type="duplicateValues" dxfId="31" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q139">
-    <cfRule type="duplicateValues" dxfId="30" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q176">
-    <cfRule type="duplicateValues" dxfId="29" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q216:Q1048576 Q140:Q146 Q177:Q209 Q211:Q212 Q48:Q71 Q1:Q27 Q118:Q138 Q40 Q74:Q116 Q42:Q45 Q29:Q38 Q148:Q175">
-    <cfRule type="duplicateValues" dxfId="28" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="R117">
-    <cfRule type="duplicateValues" dxfId="27" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="R173">
-    <cfRule type="duplicateValues" dxfId="26" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="R216:R1048576 R174:R212 R1:R38 R118:R146 R40 R73:R116 R42:R71 R148:R172">
-    <cfRule type="duplicateValues" dxfId="25" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="S88:T88 S97:T97 S102:T102 S104:T104 S111:T111 S115:T115 S120:T120 S127:T127 S130:T130 S133:T133 S145:T145 S156:T157 S165:T165 S174:T174">
-    <cfRule type="expression" dxfId="24" priority="29">
+    <cfRule type="expression" dxfId="22" priority="29">
       <formula>$S88=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X110">
-    <cfRule type="duplicateValues" dxfId="23" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC1:AC1048576 AI19:AI1048576">
-    <cfRule type="expression" dxfId="22" priority="34">
+    <cfRule type="expression" dxfId="20" priority="34">
       <formula>$AD1="ko"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD2:AD76 AA2:AA191">
-    <cfRule type="cellIs" dxfId="21" priority="35" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="35" operator="equal">
       <formula>"ko"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="36" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="36" operator="equal">
       <formula>"ok"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI1">
-    <cfRule type="expression" dxfId="19" priority="33">
+    <cfRule type="expression" dxfId="17" priority="33">
       <formula>$AD1="ko"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AJ2:AJ13">
-    <cfRule type="cellIs" dxfId="18" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="31" operator="equal">
       <formula>"ko"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="32" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="32" operator="equal">
       <formula>"ok"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AQ11:AQ21">
-    <cfRule type="duplicateValues" dxfId="16" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="AV2:AV21 AV25:AV29">
-    <cfRule type="cellIs" dxfId="15" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="6" operator="equal">
       <formula>"Estudios primarios"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="7" operator="equal">
       <formula>"Estudios secundarios"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW2:AW21 AW25:AW29">
-    <cfRule type="cellIs" dxfId="13" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="11" priority="5" operator="lessThan">
       <formula>21</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AY2:AY21">
-    <cfRule type="cellIs" dxfId="12" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="4" operator="equal">
       <formula>"NOT VALID"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AY25:AY29">
-    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
       <formula>"NOT VALID"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15053,7 +15276,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BR2:BR51">
-    <cfRule type="cellIs" dxfId="10" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="11" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15090,7 +15313,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{451DC71D-A65B-4AC5-B117-130613ABA0E8}">
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="71.42578125" style="25" bestFit="1" customWidth="1"/>
@@ -15643,8 +15866,8 @@
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
-        <v>74</v>
+      <c r="A21" t="s">
+        <v>559</v>
       </c>
       <c r="B21" s="7" t="str">
         <f>VLOOKUP(A21,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
@@ -15671,11 +15894,11 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B22" s="7" t="str">
         <f>VLOOKUP(A22,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>NEURO MKT</v>
+        <v>MKT EC</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>8</v>
@@ -15687,22 +15910,22 @@
         <v>55</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H22" s="10" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>551</v>
+        <v>78</v>
       </c>
       <c r="B23" s="7" t="str">
         <f>VLOOKUP(A23,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>DERECHO DIG.</v>
+        <v>NEURO MKT</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>8</v>
@@ -15714,22 +15937,22 @@
         <v>55</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>552</v>
+        <v>79</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>553</v>
+        <v>80</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>554</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>82</v>
+        <v>551</v>
       </c>
       <c r="B24" s="7" t="str">
         <f>VLOOKUP(A24,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>VENTAS</v>
+        <v>DERECHO DIG.</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>8</v>
@@ -15741,22 +15964,22 @@
         <v>55</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>83</v>
+        <v>552</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>84</v>
+        <v>553</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>85</v>
+        <v>554</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="B25" s="7" t="str">
         <f>VLOOKUP(A25,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>DERECHO</v>
+        <v>VENTAS</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>8</v>
@@ -15764,26 +15987,26 @@
       <c r="D25" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E25" s="14" t="s">
-        <v>87</v>
+      <c r="E25" s="13" t="s">
+        <v>55</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="B26" s="7" t="str">
         <f>VLOOKUP(A26,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>SALUD</v>
+        <v>DERECHO</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>8</v>
@@ -15795,22 +16018,22 @@
         <v>87</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>91</v>
+        <v>42</v>
       </c>
       <c r="B27" s="7" t="str">
         <f>VLOOKUP(A27,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>RSC</v>
+        <v>SALUD</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>8</v>
@@ -15822,22 +16045,22 @@
         <v>87</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>92</v>
+        <v>43</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>93</v>
+        <v>44</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>93</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B28" s="7" t="str">
         <f>VLOOKUP(A28,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>SOSTEN</v>
+        <v>RSC</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>8</v>
@@ -15849,22 +16072,22 @@
         <v>87</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="B29" s="7" t="str">
         <f>VLOOKUP(A29,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>CIBER</v>
+        <v>SOSTEN</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>8</v>
@@ -15876,22 +16099,22 @@
         <v>87</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B30" s="7" t="str">
         <f>VLOOKUP(A30,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>GDATA</v>
+        <v>CIBER</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>8</v>
@@ -15903,22 +16126,22 @@
         <v>87</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="H30" s="10" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B31" s="7" t="str">
         <f>VLOOKUP(A31,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>IA</v>
+        <v>GDATA</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>8</v>
@@ -15930,22 +16153,22 @@
         <v>87</v>
       </c>
       <c r="F31" s="10" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B32" s="7" t="str">
         <f>VLOOKUP(A32,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>PM ESP</v>
+        <v>IA</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>8</v>
@@ -15957,22 +16180,22 @@
         <v>87</v>
       </c>
       <c r="F32" s="10" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="H32" s="10" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B33" s="7" t="str">
         <f>VLOOKUP(A33,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>SISTEM</v>
+        <v>PM ESP</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>8</v>
@@ -15984,22 +16207,22 @@
         <v>87</v>
       </c>
       <c r="F33" s="10" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="15" t="s">
-        <v>120</v>
+      <c r="A34" s="12" t="s">
+        <v>116</v>
       </c>
       <c r="B34" s="7" t="str">
         <f>VLOOKUP(A34,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>FULL</v>
+        <v>SISTEM</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>8</v>
@@ -16011,18 +16234,18 @@
         <v>87</v>
       </c>
       <c r="F34" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="12" t="s">
-        <v>124</v>
+      <c r="A35" s="15" t="s">
+        <v>120</v>
       </c>
       <c r="B35" s="7" t="str">
         <f>VLOOKUP(A35,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
@@ -16048,12 +16271,12 @@
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="15" t="s">
-        <v>125</v>
+      <c r="A36" s="12" t="s">
+        <v>124</v>
       </c>
       <c r="B36" s="7" t="str">
         <f>VLOOKUP(A36,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>DEVOPS</v>
+        <v>FULL</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>8</v>
@@ -16065,22 +16288,22 @@
         <v>87</v>
       </c>
       <c r="F36" s="10" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="G36" s="11" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="H36" s="10" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B37" s="7" t="str">
         <f>VLOOKUP(A37,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>BIG DATA</v>
+        <v>DEVOPS</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>8</v>
@@ -16092,52 +16315,52 @@
         <v>87</v>
       </c>
       <c r="F37" s="10" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="12" t="s">
-        <v>133</v>
+      <c r="A38" s="15" t="s">
+        <v>129</v>
       </c>
       <c r="B38" s="7" t="str">
         <f>VLOOKUP(A38,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>IBM ENG</v>
+        <v>BIG DATA</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="E38" s="16" t="s">
-        <v>135</v>
+        <v>9</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>87</v>
       </c>
       <c r="F38" s="10" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B39" s="7" t="str">
         <f>VLOOKUP(A39,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>EMBA ENG</v>
+        <v>IBM ENG</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>139</v>
+        <v>8</v>
       </c>
       <c r="D39" s="8" t="s">
         <v>134</v>
@@ -16146,22 +16369,22 @@
         <v>135</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="17" t="s">
-        <v>142</v>
+      <c r="A40" s="12" t="s">
+        <v>138</v>
       </c>
       <c r="B40" s="7" t="str">
         <f>VLOOKUP(A40,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>RSC ENG</v>
+        <v>EMBA ENG</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>139</v>
@@ -16173,25 +16396,25 @@
         <v>135</v>
       </c>
       <c r="F40" s="10" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="H40" s="11" t="s">
-        <v>144</v>
+        <v>140</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="12" t="s">
-        <v>145</v>
+      <c r="A41" s="17" t="s">
+        <v>142</v>
       </c>
       <c r="B41" s="7" t="str">
         <f>VLOOKUP(A41,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>PM ENG</v>
+        <v>RSC ENG</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>8</v>
+        <v>139</v>
       </c>
       <c r="D41" s="8" t="s">
         <v>134</v>
@@ -16200,22 +16423,22 @@
         <v>135</v>
       </c>
       <c r="F41" s="10" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="H41" s="10" t="s">
-        <v>148</v>
+        <v>144</v>
+      </c>
+      <c r="H41" s="11" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="18" t="s">
-        <v>149</v>
+      <c r="A42" s="12" t="s">
+        <v>145</v>
       </c>
       <c r="B42" s="7" t="str">
         <f>VLOOKUP(A42,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>MKT EC ENG</v>
+        <v>PM ENG</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>8</v>
@@ -16227,22 +16450,22 @@
         <v>135</v>
       </c>
       <c r="F42" s="10" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="H42" s="11" t="s">
-        <v>151</v>
+        <v>147</v>
+      </c>
+      <c r="H42" s="10" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="15" t="s">
-        <v>152</v>
+      <c r="A43" s="18" t="s">
+        <v>149</v>
       </c>
       <c r="B43" s="7" t="str">
         <f>VLOOKUP(A43,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>SUPPLY ENG</v>
+        <v>MKT EC ENG</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>8</v>
@@ -16254,49 +16477,49 @@
         <v>135</v>
       </c>
       <c r="F43" s="10" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="H43" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
+      </c>
+      <c r="H43" s="11" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="12" t="s">
-        <v>156</v>
+      <c r="A44" s="15" t="s">
+        <v>152</v>
       </c>
       <c r="B44" s="7" t="str">
         <f>VLOOKUP(A44,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>EMBA ESP</v>
+        <v>SUPPLY ENG</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>139</v>
+        <v>8</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="E44" s="19" t="s">
-        <v>157</v>
+        <v>134</v>
+      </c>
+      <c r="E44" s="16" t="s">
+        <v>135</v>
       </c>
       <c r="F44" s="10" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="G44" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="H44" s="10" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B45" s="7" t="str">
         <f>VLOOKUP(A45,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>GMBA</v>
+        <v>EMBA ESP</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>139</v>
@@ -16308,79 +16531,97 @@
         <v>157</v>
       </c>
       <c r="F45" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="G45" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="H45" s="10" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="12" t="s">
         <v>160</v>
-      </c>
-      <c r="G45" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="H45" s="10" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="20" t="s">
-        <v>162</v>
       </c>
       <c r="B46" s="7" t="str">
         <f>VLOOKUP(A46,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
+        <v>GMBA</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E46" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="F46" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="G46" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="H46" s="10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="B47" s="7" t="str">
+        <f>VLOOKUP(A47,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
         <v>TMBA</v>
       </c>
-      <c r="C46" s="21" t="s">
+      <c r="C47" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="D46" s="21" t="s">
+      <c r="D47" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="E46" s="22" t="s">
+      <c r="E47" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="F46" s="23" t="s">
+      <c r="F47" s="23" t="s">
         <v>162</v>
       </c>
-      <c r="G46" s="24" t="s">
+      <c r="G47" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="H46" s="10" t="s">
+      <c r="H47" s="10" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E48"/>
-      <c r="F48"/>
-      <c r="G48"/>
-      <c r="H48"/>
+    <row r="49" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E49"/>
+      <c r="F49"/>
+      <c r="G49"/>
+      <c r="H49"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A20">
-    <cfRule type="duplicateValues" dxfId="9" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="8"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="9"/>
+  <conditionalFormatting sqref="A3">
+    <cfRule type="duplicateValues" dxfId="7" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A41:A46 A21:A22 A11:A19 A2:B2 A24:A39 A4:A9 B3:B46">
-    <cfRule type="duplicateValues" dxfId="4" priority="10"/>
+  <conditionalFormatting sqref="A20:A21">
+    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="9"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A23">
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+  <conditionalFormatting sqref="A24">
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A3">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  <conditionalFormatting sqref="A42:A47 A22:A23 A11:A19 A2:B2 A25:A40 A4:A9 B3:B47">
+    <cfRule type="duplicateValues" dxfId="0" priority="10"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="396b9688-3d64-4f4f-b40d-59fd809f50b1" xsi:nil="true"/>
@@ -16391,9 +16632,18 @@
 </p:properties>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A62BD1A1B5CAC249A95BCCCA1576DD25" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ac690216a3feb446896882bf9e857d22">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e4f8e1ef-7590-4615-a0b0-41d92864fb7e" xmlns:ns3="396b9688-3d64-4f4f-b40d-59fd809f50b1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fc1e276ee4a1c4eeb2be670671426ef6" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A62BD1A1B5CAC249A95BCCCA1576DD25" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="95d80e3e9b41a0cd0f31651385762a39">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e4f8e1ef-7590-4615-a0b0-41d92864fb7e" xmlns:ns3="396b9688-3d64-4f4f-b40d-59fd809f50b1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0c785e827d86c3245c0f7c251e0c72c1" ns2:_="" ns3:_="">
     <xsd:import namespace="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
     <xsd:import namespace="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
     <xsd:element name="properties">
@@ -16627,14 +16877,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42E1AB7D-C01B-4FFE-9B42-D6ED241A40A7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C8CB7F0-A062-495C-8CF5-1C769026B7CB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -16645,21 +16887,14 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B0FCCB90-18EA-419E-8607-3992FA6F6F4B}">
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42E1AB7D-C01B-4FFE-9B42-D6ED241A40A7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
-    <ds:schemaRef ds:uri="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A732D84D-91B4-4450-ADE6-4641CDFC36C8}"/>
 </file>
</xml_diff>

<commit_message>
Correcciones A-M-S y programas activos
</commit_message>
<xml_diff>
--- a/Areas_Paises.xlsx
+++ b/Areas_Paises.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta.sharepoint.com/sites/BIPOWER/Shared Documents/General/Distribución Atenea/Codigos/Distribución OBS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{A8E03CFD-D3C2-4BD9-85BF-A581898274A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{303007D5-4197-4F40-AB0E-69720AB92626}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{A8E03CFD-D3C2-4BD9-85BF-A581898274A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6876B883-8758-4835-B59E-F237D4C9A858}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{996CFF7E-4120-45EC-B5A3-4D8213062A4C}"/>
   </bookViews>
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Paises!$P$1:$V$225</definedName>
     <definedName name="PAISES">Paises!$A$1:$B$17</definedName>
     <definedName name="PILAR">Paises!$AF$1:$AG$18</definedName>
-    <definedName name="PROGRAMAS">Areas!$A$1:$G$47</definedName>
+    <definedName name="PROGRAMAS">Areas!$A$1:$G$48</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1440" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1447" uniqueCount="561">
   <si>
     <t>PROGRAMA</t>
   </si>
@@ -1726,6 +1726,9 @@
   </si>
   <si>
     <t>Máster de Formación Permanente en Marketing Digital, E-commerce e Inteligencia Artificial</t>
+  </si>
+  <si>
+    <t>Máster en Transformación Digital</t>
   </si>
 </sst>
 </file>
@@ -15313,7 +15316,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{451DC71D-A65B-4AC5-B117-130613ABA0E8}">
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="71.42578125" style="25" bestFit="1" customWidth="1"/>
@@ -15597,7 +15600,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>46</v>
+        <v>560</v>
       </c>
       <c r="B11" s="7" t="str">
         <f>VLOOKUP(A11,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
@@ -15624,11 +15627,11 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B12" s="7" t="str">
         <f>VLOOKUP(A12,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>OPER</v>
+        <v>TR DIGI</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>8</v>
@@ -15640,22 +15643,22 @@
         <v>10</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>98</v>
+        <v>50</v>
       </c>
       <c r="B13" s="7" t="str">
         <f>VLOOKUP(A13,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>BI</v>
+        <v>OPER</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>8</v>
@@ -15667,18 +15670,18 @@
         <v>10</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>99</v>
+        <v>51</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>100</v>
+        <v>52</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>100</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>101</v>
+      <c r="A14" s="12" t="s">
+        <v>98</v>
       </c>
       <c r="B14" s="7" t="str">
         <f>VLOOKUP(A14,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
@@ -15704,12 +15707,12 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
-        <v>86</v>
+      <c r="A15" s="6" t="s">
+        <v>101</v>
       </c>
       <c r="B15" s="7" t="str">
         <f>VLOOKUP(A15,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>PROD</v>
+        <v>BI</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>8</v>
@@ -15721,22 +15724,22 @@
         <v>10</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="B16" s="7" t="str">
         <f>VLOOKUP(A16,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>BRAND</v>
+        <v>PROD</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>8</v>
@@ -15744,26 +15747,26 @@
       <c r="D16" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E16" s="13" t="s">
-        <v>55</v>
+      <c r="E16" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>57</v>
+        <v>89</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>58</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B17" s="7" t="str">
         <f>VLOOKUP(A17,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>COACH</v>
+        <v>BRAND</v>
       </c>
       <c r="C17" s="8" t="s">
         <v>8</v>
@@ -15775,22 +15778,22 @@
         <v>55</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B18" s="7" t="str">
         <f>VLOOKUP(A18,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>CX</v>
+        <v>COACH</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>8</v>
@@ -15802,22 +15805,22 @@
         <v>55</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="B19" s="7" t="str">
         <f>VLOOKUP(A19,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>MKT GC</v>
+        <v>CX</v>
       </c>
       <c r="C19" s="8" t="s">
         <v>8</v>
@@ -15829,22 +15832,22 @@
         <v>55</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="93" t="s">
-        <v>550</v>
+      <c r="A20" s="12" t="s">
+        <v>70</v>
       </c>
       <c r="B20" s="7" t="str">
         <f>VLOOKUP(A20,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>MKT EC</v>
+        <v>MKT GC</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>8</v>
@@ -15856,18 +15859,18 @@
         <v>55</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="H20" s="10" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>559</v>
+      <c r="A21" s="93" t="s">
+        <v>550</v>
       </c>
       <c r="B21" s="7" t="str">
         <f>VLOOKUP(A21,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
@@ -15893,8 +15896,8 @@
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
-        <v>74</v>
+      <c r="A22" t="s">
+        <v>559</v>
       </c>
       <c r="B22" s="7" t="str">
         <f>VLOOKUP(A22,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
@@ -15921,11 +15924,11 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B23" s="7" t="str">
         <f>VLOOKUP(A23,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>NEURO MKT</v>
+        <v>MKT EC</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>8</v>
@@ -15937,22 +15940,22 @@
         <v>55</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>551</v>
+        <v>78</v>
       </c>
       <c r="B24" s="7" t="str">
         <f>VLOOKUP(A24,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>DERECHO DIG.</v>
+        <v>NEURO MKT</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>8</v>
@@ -15964,22 +15967,22 @@
         <v>55</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>552</v>
+        <v>79</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>553</v>
+        <v>80</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>554</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>82</v>
+        <v>551</v>
       </c>
       <c r="B25" s="7" t="str">
         <f>VLOOKUP(A25,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>VENTAS</v>
+        <v>DERECHO DIG.</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>8</v>
@@ -15991,22 +15994,22 @@
         <v>55</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>83</v>
+        <v>552</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>84</v>
+        <v>553</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>85</v>
+        <v>554</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="B26" s="7" t="str">
         <f>VLOOKUP(A26,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>DERECHO</v>
+        <v>VENTAS</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>8</v>
@@ -16014,26 +16017,26 @@
       <c r="D26" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E26" s="14" t="s">
-        <v>87</v>
+      <c r="E26" s="13" t="s">
+        <v>55</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="B27" s="7" t="str">
         <f>VLOOKUP(A27,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>SALUD</v>
+        <v>DERECHO</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>8</v>
@@ -16045,22 +16048,22 @@
         <v>87</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>91</v>
+        <v>42</v>
       </c>
       <c r="B28" s="7" t="str">
         <f>VLOOKUP(A28,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>RSC</v>
+        <v>SALUD</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>8</v>
@@ -16072,22 +16075,22 @@
         <v>87</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>92</v>
+        <v>43</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>93</v>
+        <v>44</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>93</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B29" s="7" t="str">
         <f>VLOOKUP(A29,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>SOSTEN</v>
+        <v>RSC</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>8</v>
@@ -16099,22 +16102,22 @@
         <v>87</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="B30" s="7" t="str">
         <f>VLOOKUP(A30,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>CIBER</v>
+        <v>SOSTEN</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>8</v>
@@ -16126,22 +16129,22 @@
         <v>87</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="H30" s="10" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B31" s="7" t="str">
         <f>VLOOKUP(A31,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>GDATA</v>
+        <v>CIBER</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>8</v>
@@ -16153,22 +16156,22 @@
         <v>87</v>
       </c>
       <c r="F31" s="10" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B32" s="7" t="str">
         <f>VLOOKUP(A32,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>IA</v>
+        <v>GDATA</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>8</v>
@@ -16180,22 +16183,22 @@
         <v>87</v>
       </c>
       <c r="F32" s="10" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H32" s="10" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B33" s="7" t="str">
         <f>VLOOKUP(A33,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>PM ESP</v>
+        <v>IA</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>8</v>
@@ -16207,22 +16210,22 @@
         <v>87</v>
       </c>
       <c r="F33" s="10" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B34" s="7" t="str">
         <f>VLOOKUP(A34,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>SISTEM</v>
+        <v>PM ESP</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>8</v>
@@ -16234,22 +16237,22 @@
         <v>87</v>
       </c>
       <c r="F34" s="10" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="15" t="s">
-        <v>120</v>
+      <c r="A35" s="12" t="s">
+        <v>116</v>
       </c>
       <c r="B35" s="7" t="str">
         <f>VLOOKUP(A35,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>FULL</v>
+        <v>SISTEM</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>8</v>
@@ -16261,18 +16264,18 @@
         <v>87</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="12" t="s">
-        <v>124</v>
+      <c r="A36" s="15" t="s">
+        <v>120</v>
       </c>
       <c r="B36" s="7" t="str">
         <f>VLOOKUP(A36,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
@@ -16298,12 +16301,12 @@
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="15" t="s">
-        <v>125</v>
+      <c r="A37" s="12" t="s">
+        <v>124</v>
       </c>
       <c r="B37" s="7" t="str">
         <f>VLOOKUP(A37,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>DEVOPS</v>
+        <v>FULL</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>8</v>
@@ -16315,22 +16318,22 @@
         <v>87</v>
       </c>
       <c r="F37" s="10" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B38" s="7" t="str">
         <f>VLOOKUP(A38,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>BIG DATA</v>
+        <v>DEVOPS</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>8</v>
@@ -16342,52 +16345,52 @@
         <v>87</v>
       </c>
       <c r="F38" s="10" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="12" t="s">
-        <v>133</v>
+      <c r="A39" s="15" t="s">
+        <v>129</v>
       </c>
       <c r="B39" s="7" t="str">
         <f>VLOOKUP(A39,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>IBM ENG</v>
+        <v>BIG DATA</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="E39" s="16" t="s">
-        <v>135</v>
+        <v>9</v>
+      </c>
+      <c r="E39" s="14" t="s">
+        <v>87</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B40" s="7" t="str">
         <f>VLOOKUP(A40,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>EMBA ENG</v>
+        <v>IBM ENG</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>139</v>
+        <v>8</v>
       </c>
       <c r="D40" s="8" t="s">
         <v>134</v>
@@ -16396,22 +16399,22 @@
         <v>135</v>
       </c>
       <c r="F40" s="10" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H40" s="10" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="17" t="s">
-        <v>142</v>
+      <c r="A41" s="12" t="s">
+        <v>138</v>
       </c>
       <c r="B41" s="7" t="str">
         <f>VLOOKUP(A41,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>RSC ENG</v>
+        <v>EMBA ENG</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>139</v>
@@ -16423,25 +16426,25 @@
         <v>135</v>
       </c>
       <c r="F41" s="10" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="H41" s="11" t="s">
-        <v>144</v>
+        <v>140</v>
+      </c>
+      <c r="H41" s="10" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="12" t="s">
-        <v>145</v>
+      <c r="A42" s="17" t="s">
+        <v>142</v>
       </c>
       <c r="B42" s="7" t="str">
         <f>VLOOKUP(A42,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>PM ENG</v>
+        <v>RSC ENG</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>8</v>
+        <v>139</v>
       </c>
       <c r="D42" s="8" t="s">
         <v>134</v>
@@ -16450,22 +16453,22 @@
         <v>135</v>
       </c>
       <c r="F42" s="10" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="H42" s="10" t="s">
-        <v>148</v>
+        <v>144</v>
+      </c>
+      <c r="H42" s="11" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="18" t="s">
-        <v>149</v>
+      <c r="A43" s="12" t="s">
+        <v>145</v>
       </c>
       <c r="B43" s="7" t="str">
         <f>VLOOKUP(A43,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>MKT EC ENG</v>
+        <v>PM ENG</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>8</v>
@@ -16477,22 +16480,22 @@
         <v>135</v>
       </c>
       <c r="F43" s="10" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="H43" s="11" t="s">
-        <v>151</v>
+        <v>147</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="15" t="s">
-        <v>152</v>
+      <c r="A44" s="18" t="s">
+        <v>149</v>
       </c>
       <c r="B44" s="7" t="str">
         <f>VLOOKUP(A44,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>SUPPLY ENG</v>
+        <v>MKT EC ENG</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>8</v>
@@ -16504,49 +16507,49 @@
         <v>135</v>
       </c>
       <c r="F44" s="10" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="G44" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="H44" s="10" t="s">
-        <v>155</v>
+        <v>151</v>
+      </c>
+      <c r="H44" s="11" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="12" t="s">
-        <v>156</v>
+      <c r="A45" s="15" t="s">
+        <v>152</v>
       </c>
       <c r="B45" s="7" t="str">
         <f>VLOOKUP(A45,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>EMBA ESP</v>
+        <v>SUPPLY ENG</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>139</v>
+        <v>8</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="E45" s="19" t="s">
-        <v>157</v>
+        <v>134</v>
+      </c>
+      <c r="E45" s="16" t="s">
+        <v>135</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="G45" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="12" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B46" s="7" t="str">
         <f>VLOOKUP(A46,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
-        <v>GMBA</v>
+        <v>EMBA ESP</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>139</v>
@@ -16558,63 +16561,90 @@
         <v>157</v>
       </c>
       <c r="F46" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="G46" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="H46" s="10" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="12" t="s">
         <v>160</v>
-      </c>
-      <c r="G46" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="H46" s="10" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A47" s="20" t="s">
-        <v>162</v>
       </c>
       <c r="B47" s="7" t="str">
         <f>VLOOKUP(A47,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
+        <v>GMBA</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E47" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="G47" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="H47" s="10" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="B48" s="7" t="str">
+        <f>VLOOKUP(A48,'[1]NORMALIZACION PROGRAMAS'!$B:$C,2,0)</f>
         <v>TMBA</v>
       </c>
-      <c r="C47" s="21" t="s">
+      <c r="C48" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="D47" s="21" t="s">
+      <c r="D48" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="E47" s="22" t="s">
+      <c r="E48" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="F47" s="23" t="s">
+      <c r="F48" s="23" t="s">
         <v>162</v>
       </c>
-      <c r="G47" s="24" t="s">
+      <c r="G48" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="H47" s="10" t="s">
+      <c r="H48" s="10" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="49" spans="5:8" x14ac:dyDescent="0.25">
-      <c r="E49"/>
-      <c r="F49"/>
-      <c r="G49"/>
-      <c r="H49"/>
+    <row r="50" spans="5:8" x14ac:dyDescent="0.25">
+      <c r="E50"/>
+      <c r="F50"/>
+      <c r="G50"/>
+      <c r="H50"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3">
     <cfRule type="duplicateValues" dxfId="7" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A20:A21">
+  <conditionalFormatting sqref="A21:A22">
     <cfRule type="duplicateValues" dxfId="6" priority="5"/>
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
     <cfRule type="duplicateValues" dxfId="4" priority="7"/>
     <cfRule type="duplicateValues" dxfId="3" priority="8"/>
     <cfRule type="duplicateValues" dxfId="2" priority="9"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A24">
+  <conditionalFormatting sqref="A25">
     <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A42:A47 A22:A23 A11:A19 A2:B2 A25:A40 A4:A9 B3:B47">
+  <conditionalFormatting sqref="A43:A48 A23:A24 A12:A20 A2:B2 A26:A41 A4:A9 B3:B48">
     <cfRule type="duplicateValues" dxfId="0" priority="10"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16622,26 +16652,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="396b9688-3d64-4f4f-b40d-59fd809f50b1" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e4f8e1ef-7590-4615-a0b0-41d92864fb7e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A62BD1A1B5CAC249A95BCCCA1576DD25" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="95d80e3e9b41a0cd0f31651385762a39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e4f8e1ef-7590-4615-a0b0-41d92864fb7e" xmlns:ns3="396b9688-3d64-4f4f-b40d-59fd809f50b1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0c785e827d86c3245c0f7c251e0c72c1" ns2:_="" ns3:_="">
     <xsd:import namespace="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
@@ -16876,13 +16886,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="396b9688-3d64-4f4f-b40d-59fd809f50b1" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e4f8e1ef-7590-4615-a0b0-41d92864fb7e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C8CB7F0-A062-495C-8CF5-1C769026B7CB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A732D84D-91B4-4450-ADE6-4641CDFC36C8}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
+    <ds:schemaRef ds:uri="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
-    <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -16896,5 +16934,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A732D84D-91B4-4450-ADE6-4641CDFC36C8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C8CB7F0-A062-495C-8CF5-1C769026B7CB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
+    <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Cambios C4 y area E
</commit_message>
<xml_diff>
--- a/Areas_Paises.xlsx
+++ b/Areas_Paises.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta.sharepoint.com/sites/BIPOWER/Shared Documents/General/Distribución Atenea/Codigos/Distribución OBS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{A8E03CFD-D3C2-4BD9-85BF-A581898274A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48F903F3-F0EA-47A0-812A-65A3C85D5C27}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:1_{A8E03CFD-D3C2-4BD9-85BF-A581898274A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D1F1FD3-0B54-4495-A00D-10024BDBB009}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-45" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{996CFF7E-4120-45EC-B5A3-4D8213062A4C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{996CFF7E-4120-45EC-B5A3-4D8213062A4C}"/>
   </bookViews>
   <sheets>
     <sheet name="Paises" sheetId="2" r:id="rId1"/>
@@ -15357,11 +15357,11 @@
     <cfRule type="duplicateValues" dxfId="19" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="AV2:AV21 AV25:AV29">
-    <cfRule type="cellIs" dxfId="18" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="7" operator="equal">
+      <formula>"Estudios secundarios"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="17" priority="6" operator="equal">
       <formula>"Estudios primarios"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="7" operator="equal">
-      <formula>"Estudios secundarios"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AW2:AW21 AW25:AW29">
@@ -15544,8 +15544,8 @@
       <c r="D4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>10</v>
+      <c r="E4" s="14" t="s">
+        <v>87</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>16</v>
@@ -15652,8 +15652,8 @@
       <c r="D8" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="9" t="s">
-        <v>10</v>
+      <c r="E8" s="14" t="s">
+        <v>87</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>32</v>
@@ -16003,8 +16003,8 @@
       <c r="D21" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E21" s="13" t="s">
-        <v>55</v>
+      <c r="E21" s="14" t="s">
+        <v>87</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>64</v>
@@ -16850,23 +16850,25 @@
     <cfRule type="duplicateValues" dxfId="3" priority="13"/>
     <cfRule type="duplicateValues" dxfId="2" priority="14"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A25:A26 A12:A14 A2:B2 A28:A43 A4:A9 A21:A22 A16:A19 A45 A47:A51 B3:B51">
+    <cfRule type="duplicateValues" dxfId="1" priority="15"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A27">
-    <cfRule type="duplicateValues" dxfId="1" priority="9"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A25:A26 A12:A14 A2:B2 A28:A43 A4:A9 A21:A22 A16:A19 A45 A47:A51 B3:B51">
-    <cfRule type="duplicateValues" dxfId="0" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="9"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="396b9688-3d64-4f4f-b40d-59fd809f50b1" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e4f8e1ef-7590-4615-a0b0-41d92864fb7e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17105,20 +17107,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="396b9688-3d64-4f4f-b40d-59fd809f50b1" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e4f8e1ef-7590-4615-a0b0-41d92864fb7e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42E1AB7D-C01B-4FFE-9B42-D6ED241A40A7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C8CB7F0-A062-495C-8CF5-1C769026B7CB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
+    <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -17143,12 +17146,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2C8CB7F0-A062-495C-8CF5-1C769026B7CB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42E1AB7D-C01B-4FFE-9B42-D6ED241A40A7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
-    <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>